<commit_message>
add tiktok publish section for demo
</commit_message>
<xml_diff>
--- a/AQUAVO_FINAL_v9.xlsx
+++ b/AQUAVO_FINAL_v9.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jaafa\Desktop\upload\FishWebClean\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F35309D-2EFB-40D5-94AA-92FE5EF25290}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D6A4F46-6F8B-4C9F-92E2-68771D718F5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1243,19 +1243,19 @@
         <v>8600</v>
       </c>
       <c r="J8" s="9">
-        <v>14300</v>
+        <v>15500</v>
       </c>
       <c r="K8" s="6">
         <f t="shared" si="2"/>
-        <v>0.39860139860139859</v>
+        <v>0.44516129032258067</v>
       </c>
       <c r="L8" s="10">
         <f t="shared" si="3"/>
-        <v>5700</v>
+        <v>6900</v>
       </c>
       <c r="M8" s="10">
         <f t="shared" si="0"/>
-        <v>28500</v>
+        <v>34500</v>
       </c>
       <c r="N8" s="7">
         <v>13.3</v>
@@ -4742,7 +4742,7 @@
       </c>
       <c r="N70" s="5">
         <f>SUM(M4:M69)</f>
-        <v>3346021</v>
+        <v>3352021</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
perf: convert images to WebP (87% smaller), add hero preload, auto-WebP paths, update DB image refs, fix products description
</commit_message>
<xml_diff>
--- a/AQUAVO_FINAL_v9.xlsx
+++ b/AQUAVO_FINAL_v9.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jaafa\Desktop\upload\FishWebClean\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D6A4F46-6F8B-4C9F-92E2-68771D718F5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{657668EC-1223-41BC-BB04-AB141203B92D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3723,19 +3723,19 @@
         <v>3587</v>
       </c>
       <c r="J52" s="9">
-        <v>6600</v>
+        <v>8000</v>
       </c>
       <c r="K52" s="6">
         <f t="shared" si="2"/>
-        <v>0.45651515151515154</v>
+        <v>0.55162500000000003</v>
       </c>
       <c r="L52" s="10">
         <f t="shared" si="3"/>
-        <v>3013</v>
+        <v>4413</v>
       </c>
       <c r="M52" s="10">
         <f t="shared" si="4"/>
-        <v>45195</v>
+        <v>66195</v>
       </c>
       <c r="N52" s="7">
         <v>54.4</v>
@@ -4742,7 +4742,7 @@
       </c>
       <c r="N70" s="5">
         <f>SUM(M4:M69)</f>
-        <v>3352021</v>
+        <v>3373021</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: guest reviews + loyalty tier badges + admin moderation workflow
</commit_message>
<xml_diff>
--- a/AQUAVO_FINAL_v9.xlsx
+++ b/AQUAVO_FINAL_v9.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jaafa\Desktop\upload\FishWebClean\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{657668EC-1223-41BC-BB04-AB141203B92D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D757B89F-9740-4374-8820-CDE2E75A7EDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -413,7 +413,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -460,6 +460,12 @@
         <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -490,7 +496,7 @@
     <xf numFmtId="44" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
@@ -543,15 +549,6 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="2"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="7" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="2"/>
     </xf>
@@ -560,6 +557,37 @@
       <alignment horizontal="center" vertical="center" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="10" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="10" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="9" fontId="7" fillId="10" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="6" fillId="10" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="2"/>
     </xf>
   </cellXfs>
@@ -889,48 +917,48 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A1" s="24" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
-      <c r="I1" s="22"/>
-      <c r="J1" s="22"/>
-      <c r="K1" s="22"/>
-      <c r="L1" s="22"/>
-      <c r="M1" s="22"/>
-      <c r="N1" s="22"/>
-      <c r="O1" s="22"/>
-      <c r="P1" s="22"/>
-      <c r="Q1" s="22"/>
-      <c r="R1" s="22"/>
+      <c r="A1" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
+      <c r="N1" s="19"/>
+      <c r="O1" s="19"/>
+      <c r="P1" s="19"/>
+      <c r="Q1" s="19"/>
+      <c r="R1" s="19"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
-      <c r="I2" s="22"/>
-      <c r="J2" s="22"/>
-      <c r="K2" s="22"/>
-      <c r="L2" s="22"/>
-      <c r="M2" s="22"/>
-      <c r="N2" s="22"/>
-      <c r="O2" s="22"/>
-      <c r="P2" s="22"/>
-      <c r="Q2" s="22"/>
-      <c r="R2" s="22"/>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19"/>
+      <c r="J2" s="19"/>
+      <c r="K2" s="19"/>
+      <c r="L2" s="19"/>
+      <c r="M2" s="19"/>
+      <c r="N2" s="19"/>
+      <c r="O2" s="19"/>
+      <c r="P2" s="19"/>
+      <c r="Q2" s="19"/>
+      <c r="R2" s="19"/>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -2262,292 +2290,292 @@
       <c r="P26" s="7"/>
       <c r="Q26" s="7"/>
     </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A27" s="3">
+    <row r="27" spans="1:17" s="31" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="22">
         <v>24</v>
       </c>
-      <c r="B27" s="13" t="s">
+      <c r="B27" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="C27" s="17" t="s">
+      <c r="C27" s="24" t="s">
         <v>45</v>
       </c>
-      <c r="D27" s="11">
+      <c r="D27" s="25">
         <v>2</v>
       </c>
-      <c r="E27" s="11">
+      <c r="E27" s="25">
         <v>6.28</v>
       </c>
-      <c r="F27" s="11">
+      <c r="F27" s="25">
         <v>9548</v>
       </c>
-      <c r="G27" s="11">
+      <c r="G27" s="25">
         <v>8132</v>
       </c>
-      <c r="H27" s="20">
+      <c r="H27" s="26">
         <v>6188</v>
       </c>
-      <c r="I27" s="8">
+      <c r="I27" s="27">
         <f>F27+G27+H27</f>
         <v>23868</v>
       </c>
-      <c r="J27" s="18">
+      <c r="J27" s="28">
         <f>31500+H27</f>
         <v>37688</v>
       </c>
-      <c r="K27" s="6">
+      <c r="K27" s="29">
         <f t="shared" si="2"/>
         <v>0.36669496922097217</v>
       </c>
-      <c r="L27" s="10">
+      <c r="L27" s="30">
         <f t="shared" si="3"/>
         <v>13820</v>
       </c>
-      <c r="M27" s="10">
+      <c r="M27" s="30">
         <f t="shared" si="4"/>
         <v>27640</v>
       </c>
-      <c r="N27" s="11">
+      <c r="N27" s="25">
         <v>22.2</v>
       </c>
-      <c r="O27" s="11">
+      <c r="O27" s="25">
         <v>17.899999999999999</v>
       </c>
-      <c r="P27" s="11">
+      <c r="P27" s="25">
         <v>30</v>
       </c>
-      <c r="Q27" s="11">
+      <c r="Q27" s="25">
         <v>550</v>
       </c>
     </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A28" s="2">
+    <row r="28" spans="1:17" s="31" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="22">
         <v>25</v>
       </c>
-      <c r="B28" s="12" t="s">
+      <c r="B28" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="C28" s="17" t="s">
+      <c r="C28" s="24" t="s">
         <v>45</v>
       </c>
-      <c r="D28" s="7">
+      <c r="D28" s="25">
         <v>2</v>
       </c>
-      <c r="E28" s="7">
+      <c r="E28" s="25">
         <v>9.73</v>
       </c>
-      <c r="F28" s="7">
+      <c r="F28" s="25">
         <v>14793</v>
       </c>
-      <c r="G28" s="7">
+      <c r="G28" s="25">
         <v>12565</v>
       </c>
-      <c r="H28" s="19">
+      <c r="H28" s="26">
         <v>8214</v>
       </c>
-      <c r="I28" s="8">
+      <c r="I28" s="27">
         <f>F28+G28+H28</f>
         <v>35572</v>
       </c>
-      <c r="J28" s="18">
+      <c r="J28" s="28">
         <f>(46250)+H28</f>
         <v>54464</v>
       </c>
-      <c r="K28" s="6">
+      <c r="K28" s="29">
         <f t="shared" si="2"/>
         <v>0.34687132784958874</v>
       </c>
-      <c r="L28" s="10">
+      <c r="L28" s="30">
         <f t="shared" si="3"/>
         <v>18892</v>
       </c>
-      <c r="M28" s="10">
+      <c r="M28" s="30">
         <f t="shared" si="4"/>
         <v>37784</v>
       </c>
-      <c r="N28" s="7">
+      <c r="N28" s="25">
         <v>22</v>
       </c>
-      <c r="O28" s="7">
+      <c r="O28" s="25">
         <v>17.7</v>
       </c>
-      <c r="P28" s="7">
+      <c r="P28" s="25">
         <v>46</v>
       </c>
-      <c r="Q28" s="7">
+      <c r="Q28" s="25">
         <v>250</v>
       </c>
     </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A29" s="3">
+    <row r="29" spans="1:17" s="31" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="22">
         <v>26</v>
       </c>
-      <c r="B29" s="13" t="s">
+      <c r="B29" s="23" t="s">
         <v>49</v>
       </c>
-      <c r="C29" s="17" t="s">
+      <c r="C29" s="24" t="s">
         <v>45</v>
       </c>
-      <c r="D29" s="11">
+      <c r="D29" s="25">
         <v>2</v>
       </c>
-      <c r="E29" s="11">
+      <c r="E29" s="25">
         <v>12.52</v>
       </c>
-      <c r="F29" s="11">
+      <c r="F29" s="25">
         <v>19032</v>
       </c>
-      <c r="G29" s="11">
+      <c r="G29" s="25">
         <v>16288</v>
       </c>
-      <c r="H29" s="11">
+      <c r="H29" s="25">
         <v>7351</v>
       </c>
-      <c r="I29" s="8">
+      <c r="I29" s="27">
         <f t="shared" ref="I29" si="5">F29+G29+H29</f>
         <v>42671</v>
       </c>
-      <c r="J29" s="18">
+      <c r="J29" s="28">
         <f>58580+H29</f>
         <v>65931</v>
       </c>
-      <c r="K29" s="6">
+      <c r="K29" s="29">
         <f t="shared" si="2"/>
         <v>0.35279307154449346</v>
       </c>
-      <c r="L29" s="10">
+      <c r="L29" s="30">
         <f t="shared" si="3"/>
         <v>23260</v>
       </c>
-      <c r="M29" s="10">
+      <c r="M29" s="30">
         <f t="shared" si="4"/>
         <v>46520</v>
       </c>
-      <c r="N29" s="11">
+      <c r="N29" s="25">
         <v>21.5</v>
       </c>
-      <c r="O29" s="11">
+      <c r="O29" s="25">
         <v>17.2</v>
       </c>
-      <c r="P29" s="11">
+      <c r="P29" s="25">
         <v>58</v>
       </c>
-      <c r="Q29" s="11">
+      <c r="Q29" s="25">
         <v>850</v>
       </c>
     </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A30" s="2">
+    <row r="30" spans="1:17" s="31" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="22">
         <v>27</v>
       </c>
-      <c r="B30" s="12" t="s">
+      <c r="B30" s="23" t="s">
         <v>50</v>
       </c>
-      <c r="C30" s="17" t="s">
+      <c r="C30" s="24" t="s">
         <v>45</v>
       </c>
-      <c r="D30" s="7">
+      <c r="D30" s="25">
         <v>2</v>
       </c>
-      <c r="E30" s="7">
+      <c r="E30" s="25">
         <v>8.59</v>
       </c>
-      <c r="F30" s="7">
+      <c r="F30" s="25">
         <v>13059</v>
       </c>
-      <c r="G30" s="7">
+      <c r="G30" s="25">
         <v>13097</v>
       </c>
-      <c r="H30" s="7">
+      <c r="H30" s="25">
         <v>5044</v>
       </c>
-      <c r="I30" s="8">
+      <c r="I30" s="27">
         <f>F30+G30+H30</f>
         <v>31200</v>
       </c>
-      <c r="J30" s="9">
+      <c r="J30" s="32">
         <f>43400+H30</f>
         <v>48444</v>
       </c>
-      <c r="K30" s="6">
+      <c r="K30" s="29">
         <f t="shared" si="2"/>
         <v>0.35595739410453309</v>
       </c>
-      <c r="L30" s="10">
+      <c r="L30" s="30">
         <f t="shared" si="3"/>
         <v>17244</v>
       </c>
-      <c r="M30" s="10">
+      <c r="M30" s="30">
         <f t="shared" si="4"/>
         <v>34488</v>
       </c>
-      <c r="N30" s="7">
+      <c r="N30" s="25">
         <v>21.4</v>
       </c>
-      <c r="O30" s="7">
+      <c r="O30" s="25">
         <v>17</v>
       </c>
-      <c r="P30" s="7">
+      <c r="P30" s="25">
         <v>43</v>
       </c>
-      <c r="Q30" s="7">
+      <c r="Q30" s="25">
         <v>400</v>
       </c>
     </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A31" s="3">
+    <row r="31" spans="1:17" s="31" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="22">
         <v>28</v>
       </c>
-      <c r="B31" s="13" t="s">
+      <c r="B31" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="C31" s="17" t="s">
+      <c r="C31" s="24" t="s">
         <v>45</v>
       </c>
-      <c r="D31" s="11">
+      <c r="D31" s="25">
         <v>2</v>
       </c>
-      <c r="E31" s="11">
+      <c r="E31" s="25">
         <v>11.55</v>
       </c>
-      <c r="F31" s="11">
+      <c r="F31" s="25">
         <v>17555</v>
       </c>
-      <c r="G31" s="11">
+      <c r="G31" s="25">
         <v>16022</v>
       </c>
-      <c r="H31" s="11">
+      <c r="H31" s="25">
         <v>6781</v>
       </c>
-      <c r="I31" s="8">
+      <c r="I31" s="27">
         <f>F31+G31+H31</f>
         <v>40358</v>
       </c>
-      <c r="J31" s="9">
+      <c r="J31" s="32">
         <v>55550</v>
       </c>
-      <c r="K31" s="6">
+      <c r="K31" s="29">
         <f t="shared" si="2"/>
         <v>0.27348334833483351</v>
       </c>
-      <c r="L31" s="10">
+      <c r="L31" s="30">
         <f t="shared" si="3"/>
         <v>15192</v>
       </c>
-      <c r="M31" s="10">
+      <c r="M31" s="30">
         <f t="shared" si="4"/>
         <v>30384</v>
       </c>
-      <c r="N31" s="11">
+      <c r="N31" s="25">
         <v>21.2</v>
       </c>
-      <c r="O31" s="11">
+      <c r="O31" s="25">
         <v>16.899999999999999</v>
       </c>
-      <c r="P31" s="11">
+      <c r="P31" s="25">
         <v>55</v>
       </c>
-      <c r="Q31" s="11">
+      <c r="Q31" s="25">
         <v>550</v>
       </c>
     </row>
@@ -4523,19 +4551,19 @@
         <v>10074</v>
       </c>
       <c r="J66" s="9">
-        <v>12300</v>
+        <v>12500</v>
       </c>
       <c r="K66" s="6">
         <f t="shared" si="2"/>
-        <v>0.18097560975609756</v>
+        <v>0.19408</v>
       </c>
       <c r="L66" s="10">
         <f t="shared" si="3"/>
-        <v>2226</v>
+        <v>2426</v>
       </c>
       <c r="M66" s="10">
         <f t="shared" si="4"/>
-        <v>22260</v>
+        <v>24260</v>
       </c>
       <c r="N66" s="7">
         <v>22.4</v>
@@ -4722,18 +4750,18 @@
       </c>
     </row>
     <row r="70" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A70" s="23" t="s">
+      <c r="A70" s="20" t="s">
         <v>88</v>
       </c>
-      <c r="B70" s="22"/>
-      <c r="C70" s="22"/>
-      <c r="D70" s="22"/>
-      <c r="E70" s="22"/>
-      <c r="F70" s="22"/>
-      <c r="G70" s="22"/>
-      <c r="H70" s="22"/>
-      <c r="I70" s="22"/>
-      <c r="J70" s="22"/>
+      <c r="B70" s="19"/>
+      <c r="C70" s="19"/>
+      <c r="D70" s="19"/>
+      <c r="E70" s="19"/>
+      <c r="F70" s="19"/>
+      <c r="G70" s="19"/>
+      <c r="H70" s="19"/>
+      <c r="I70" s="19"/>
+      <c r="J70" s="19"/>
       <c r="K70" s="4">
         <v>6412350</v>
       </c>
@@ -4742,7 +4770,7 @@
       </c>
       <c r="N70" s="5">
         <f>SUM(M4:M69)</f>
-        <v>3373021</v>
+        <v>3375021</v>
       </c>
     </row>
   </sheetData>

</xml_diff>